<commit_message>
feature: period type mission 추가. fix: builder 오류 수정. (group key 버그 수정)
</commit_message>
<xml_diff>
--- a/input/Domains/Game/MetaTable.xlsx
+++ b/input/Domains/Game/MetaTable.xlsx
@@ -8,25 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7FD1E2B-24F2-FE41-81CC-7399AF42B90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA78E311-7903-A249-B9DF-F6A83404C22A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1780" yWindow="500" windowWidth="37020" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1380" yWindow="500" windowWidth="37020" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MESSAGE_META" sheetId="1" r:id="rId1"/>
-    <sheet name="MISSION" sheetId="2" r:id="rId2"/>
-    <sheet name="ACHIEVE_ONCE" sheetId="3" r:id="rId3"/>
-    <sheet name="ACHIEVE_PASS" sheetId="4" r:id="rId4"/>
-    <sheet name="LEADERBOARD" sheetId="5" r:id="rId5"/>
-    <sheet name="LEADERBOARD_REWARD" sheetId="6" r:id="rId6"/>
-    <sheet name="ADVERTISE" sheetId="7" r:id="rId7"/>
+    <sheet name="MISSION_DAILY" sheetId="2" r:id="rId2"/>
+    <sheet name="MISSION_PERIOD" sheetId="3" r:id="rId3"/>
+    <sheet name="ACHIEVE_ONCE" sheetId="4" r:id="rId4"/>
+    <sheet name="ACHIEVE_PASS" sheetId="5" r:id="rId5"/>
+    <sheet name="LEADERBOARD" sheetId="6" r:id="rId6"/>
+    <sheet name="LEADERBOARD_REWARD" sheetId="7" r:id="rId7"/>
+    <sheet name="ADVERTISE" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="172">
   <si>
     <t>messageId</t>
   </si>
@@ -166,9 +167,6 @@
     <t>missionId</t>
   </si>
   <si>
-    <t>missionType</t>
-  </si>
-  <si>
     <t>isActive</t>
   </si>
   <si>
@@ -190,9 +188,6 @@
     <t>rewardGroupId</t>
   </si>
   <si>
-    <t>MISSION_TYPE</t>
-  </si>
-  <si>
     <t>bool</t>
   </si>
   <si>
@@ -217,7 +212,7 @@
     <t>UI 정렬 기준 값 (1부터 시작). daily selected runtime은 이 값을 기준으로 정렬 후 0-based Index를 부여한다.</t>
   </si>
   <si>
-    <t>MESSAGE.messageId</t>
+    <t>MESSAGE_META.messageId</t>
   </si>
   <si>
     <t>NONE/EQ/GTE/LTE</t>
@@ -232,9 +227,6 @@
     <t>mission_day_001</t>
   </si>
   <si>
-    <t>DAY</t>
-  </si>
-  <si>
     <t>GTE</t>
   </si>
   <si>
@@ -263,6 +255,12 @@
   </si>
   <si>
     <t>reward_mission_day_005</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>활성화 day (1~7). day=1 즉시 활성화, day=n은 (n-1)일 후 활성화</t>
   </si>
   <si>
     <t>index</t>
@@ -502,22 +500,53 @@
   </si>
   <si>
     <t>ad_rewarded_001</t>
+  </si>
+  <si>
+    <t>REWARDED</t>
+  </si>
+  <si>
+    <t>reward_chest_001</t>
+  </si>
+  <si>
+    <t>ca-app-pub-3442497187818240/5199204671</t>
+  </si>
+  <si>
+    <t>app_open_launch</t>
+  </si>
+  <si>
+    <t>APP_OPEN</t>
+  </si>
+  <si>
+    <t>mission_period_01_001</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>REWARDED</t>
-  </si>
-  <si>
-    <t>reward_chest_001</t>
-  </si>
-  <si>
-    <t>ca-app-pub-3442497187818240/5199204671</t>
-  </si>
-  <si>
-    <t>app_open_launch</t>
-  </si>
-  <si>
-    <t>APP_OPEN</t>
+    <t>mission_period_01_002</t>
+  </si>
+  <si>
+    <t>mission_period_01_003</t>
+  </si>
+  <si>
+    <t>mission_period_01_004</t>
+  </si>
+  <si>
+    <t>mission_period_01_005</t>
+  </si>
+  <si>
+    <t>mission_period_02_001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>mission_period_02_002</t>
+  </si>
+  <si>
+    <t>mission_period_02_003</t>
+  </si>
+  <si>
+    <t>mission_period_02_004</t>
+  </si>
+  <si>
+    <t>mission_period_02_005</t>
   </si>
 </sst>
 </file>
@@ -1133,22 +1162,20 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C20" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -1173,288 +1200,588 @@
       <c r="H1" t="s">
         <v>52</v>
       </c>
-      <c r="I1" t="s">
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
         <v>54</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
         <v>55</v>
       </c>
-      <c r="D2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>56</v>
       </c>
-      <c r="F2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>57</v>
-      </c>
       <c r="H2" t="s">
-        <v>58</v>
-      </c>
-      <c r="I2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
         <v>59</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>60</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>61</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>62</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>63</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>64</v>
       </c>
-      <c r="H4" t="s">
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
         <v>65</v>
       </c>
-      <c r="I4" t="s">
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5" t="s">
         <v>67</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
         <v>68</v>
       </c>
-      <c r="C5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6" t="s">
         <v>69</v>
       </c>
-      <c r="H5">
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8">
         <v>4</v>
       </c>
-      <c r="I5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" t="b">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G6" t="s">
-        <v>69</v>
-      </c>
-      <c r="H6">
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8">
         <v>5</v>
       </c>
-      <c r="I6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
+      <c r="H8" t="s">
         <v>73</v>
       </c>
-      <c r="B7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" t="b">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>3</v>
-      </c>
-      <c r="F7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H7">
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9">
         <v>5</v>
       </c>
-      <c r="I7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9">
+        <v>5</v>
+      </c>
+      <c r="H9" t="s">
         <v>75</v>
-      </c>
-      <c r="B8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C8" t="b">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>4</v>
-      </c>
-      <c r="F8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G8" t="s">
-        <v>69</v>
-      </c>
-      <c r="H8">
-        <v>5</v>
-      </c>
-      <c r="I8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>5</v>
-      </c>
-      <c r="F9" t="s">
-        <v>30</v>
-      </c>
-      <c r="G9" t="s">
-        <v>69</v>
-      </c>
-      <c r="H9">
-        <v>5</v>
-      </c>
-      <c r="I9" t="s">
-        <v>78</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:I9" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.28515625" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9">
+        <v>5</v>
+      </c>
+      <c r="G9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F10">
+        <v>5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>168</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11">
+        <v>5</v>
+      </c>
+      <c r="G11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" t="s">
+        <v>66</v>
+      </c>
+      <c r="F12">
+        <v>5</v>
+      </c>
+      <c r="G12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>170</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F13">
+        <v>5</v>
+      </c>
+      <c r="G13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>171</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14">
+        <v>5</v>
+      </c>
+      <c r="G14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" t="s">
         <v>79</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
         <v>80</v>
       </c>
-      <c r="C1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
         <v>81</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H1" t="s">
         <v>49</v>
       </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1" t="s">
+        <v>51</v>
+      </c>
+      <c r="K1" t="s">
+        <v>52</v>
+      </c>
+      <c r="L1" t="s">
         <v>83</v>
       </c>
-      <c r="H1" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1" t="s">
-        <v>51</v>
-      </c>
-      <c r="J1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K1" t="s">
-        <v>53</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>84</v>
-      </c>
-      <c r="M1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="H2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" t="s">
         <v>55</v>
       </c>
-      <c r="D2" t="s">
+      <c r="J2" t="s">
         <v>56</v>
-      </c>
-      <c r="E2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" t="s">
-        <v>57</v>
-      </c>
-      <c r="J2" t="s">
-        <v>58</v>
       </c>
       <c r="K2" t="s">
         <v>3</v>
@@ -1471,36 +1798,36 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
         <v>87</v>
       </c>
-      <c r="C4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>88</v>
       </c>
-      <c r="E4" t="s">
+      <c r="I4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J4" t="s">
         <v>89</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>64</v>
       </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>90</v>
       </c>
-      <c r="K4" t="s">
-        <v>66</v>
-      </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>91</v>
-      </c>
-      <c r="M4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1508,7 +1835,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -1523,16 +1850,16 @@
         <v>10</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J5">
         <v>10</v>
       </c>
       <c r="K5" t="s">
+        <v>93</v>
+      </c>
+      <c r="M5" t="s">
         <v>94</v>
-      </c>
-      <c r="M5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1540,7 +1867,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -1555,13 +1882,13 @@
         <v>10</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J6">
         <v>40</v>
       </c>
       <c r="K6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1569,7 +1896,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -1584,13 +1911,13 @@
         <v>10</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J7">
         <v>200</v>
       </c>
       <c r="K7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1598,7 +1925,7 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
@@ -1613,13 +1940,13 @@
         <v>10</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J8">
         <v>1000</v>
       </c>
       <c r="K8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1627,7 +1954,7 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -1642,13 +1969,13 @@
         <v>10</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J9">
         <v>5000</v>
       </c>
       <c r="K9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1656,7 +1983,7 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
@@ -1671,19 +1998,19 @@
         <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H10" t="s">
         <v>13</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J10">
         <v>100</v>
       </c>
       <c r="K10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1691,7 +2018,7 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
@@ -1706,19 +2033,19 @@
         <v>13</v>
       </c>
       <c r="G11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H11" t="s">
         <v>15</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J11">
         <v>100</v>
       </c>
       <c r="K11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1726,7 +2053,7 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" t="b">
         <v>1</v>
@@ -1741,19 +2068,19 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H12" t="s">
         <v>17</v>
       </c>
       <c r="I12" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J12">
         <v>100</v>
       </c>
       <c r="K12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1761,7 +2088,7 @@
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C13" t="b">
         <v>1</v>
@@ -1776,100 +2103,97 @@
         <v>17</v>
       </c>
       <c r="G13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H13" t="s">
         <v>19</v>
       </c>
       <c r="I13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J13">
         <v>100</v>
       </c>
       <c r="K13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:M13" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" t="s">
         <v>79</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
         <v>80</v>
       </c>
-      <c r="C1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D1" t="s">
-        <v>81</v>
-      </c>
       <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H1" t="s">
         <v>49</v>
       </c>
-      <c r="F1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G1" t="s">
-        <v>106</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>50</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>51</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>52</v>
-      </c>
-      <c r="K1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J2" t="s">
         <v>56</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" t="s">
-        <v>57</v>
-      </c>
-      <c r="J2" t="s">
-        <v>58</v>
       </c>
       <c r="K2" t="s">
         <v>3</v>
@@ -1880,36 +2204,36 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
         <v>87</v>
       </c>
-      <c r="C4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>88</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J4" t="s">
         <v>89</v>
       </c>
-      <c r="F4" t="s">
-        <v>107</v>
-      </c>
-      <c r="G4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>64</v>
-      </c>
-      <c r="J4" t="s">
-        <v>90</v>
-      </c>
-      <c r="K4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1917,22 +2241,22 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
         <v>109</v>
       </c>
-      <c r="C5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>110</v>
-      </c>
       <c r="K5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1940,7 +2264,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -1952,10 +2276,10 @@
         <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1963,22 +2287,22 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
         <v>109</v>
       </c>
-      <c r="C7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>3</v>
-      </c>
-      <c r="E7">
-        <v>3</v>
-      </c>
-      <c r="F7" t="s">
-        <v>110</v>
-      </c>
       <c r="K7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1986,7 +2310,7 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
@@ -1998,10 +2322,10 @@
         <v>4</v>
       </c>
       <c r="F8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -2009,7 +2333,7 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -2021,10 +2345,10 @@
         <v>5</v>
       </c>
       <c r="F9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2032,25 +2356,25 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>109</v>
+      </c>
+      <c r="G10" t="s">
         <v>111</v>
       </c>
-      <c r="C10" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>110</v>
-      </c>
-      <c r="G10" t="s">
-        <v>112</v>
-      </c>
       <c r="K10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -2058,7 +2382,7 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
@@ -2070,13 +2394,13 @@
         <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2084,25 +2408,25 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G12" t="s">
         <v>111</v>
       </c>
-      <c r="C12" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12">
-        <v>3</v>
-      </c>
-      <c r="E12">
-        <v>3</v>
-      </c>
-      <c r="F12" t="s">
-        <v>110</v>
-      </c>
-      <c r="G12" t="s">
-        <v>112</v>
-      </c>
       <c r="K12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2110,7 +2434,7 @@
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C13" t="b">
         <v>1</v>
@@ -2122,13 +2446,13 @@
         <v>4</v>
       </c>
       <c r="F13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2136,7 +2460,7 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C14" t="b">
         <v>1</v>
@@ -2148,50 +2472,47 @@
         <v>5</v>
       </c>
       <c r="F14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:K14" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E1" t="s">
         <v>114</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>115</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>116</v>
-      </c>
-      <c r="G1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -2199,13 +2520,13 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
@@ -2224,30 +2545,30 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
         <v>119</v>
       </c>
-      <c r="B4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>120</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>121</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>122</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>123</v>
-      </c>
-      <c r="G4" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B5" t="b">
         <v>1</v>
@@ -2256,58 +2577,55 @@
         <v>32</v>
       </c>
       <c r="D5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5" t="s">
         <v>126</v>
-      </c>
-      <c r="E5" t="s">
-        <v>110</v>
-      </c>
-      <c r="G5" t="s">
-        <v>127</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:G5" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" t="s">
         <v>128</v>
       </c>
-      <c r="D1" t="s">
-        <v>129</v>
-      </c>
       <c r="E1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
@@ -2318,24 +2636,24 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" t="s">
         <v>131</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>132</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>133</v>
       </c>
-      <c r="D4" t="s">
-        <v>134</v>
-      </c>
       <c r="E4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2343,7 +2661,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -2352,7 +2670,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2360,7 +2678,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -2369,50 +2687,47 @@
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:E6" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFEC218C-276E-2841-A963-2BD017001F28}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -2420,22 +2735,22 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>143</v>
-      </c>
       <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>3</v>
@@ -2459,42 +2774,42 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -2509,13 +2824,13 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="C6" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -2530,16 +2845,16 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="E7" s="1" t="b">
         <v>1</v>
@@ -2551,19 +2866,19 @@
         <v>0</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="C8" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>

</xml_diff>

<commit_message>
feature: Version check 기능 추가. refactor: 클래스 이름 정리.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/MetaTable.xlsx
+++ b/input/Domains/Game/MetaTable.xlsx
@@ -8,26 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA78E311-7903-A249-B9DF-F6A83404C22A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D03233A-D2C9-134A-AA68-2C0E24318E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="500" windowWidth="37020" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1380" yWindow="500" windowWidth="37020" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MESSAGE_META" sheetId="1" r:id="rId1"/>
-    <sheet name="MISSION_DAILY" sheetId="2" r:id="rId2"/>
-    <sheet name="MISSION_PERIOD" sheetId="3" r:id="rId3"/>
-    <sheet name="ACHIEVE_ONCE" sheetId="4" r:id="rId4"/>
-    <sheet name="ACHIEVE_PASS" sheetId="5" r:id="rId5"/>
-    <sheet name="LEADERBOARD" sheetId="6" r:id="rId6"/>
-    <sheet name="LEADERBOARD_REWARD" sheetId="7" r:id="rId7"/>
-    <sheet name="ADVERTISE" sheetId="8" r:id="rId8"/>
+    <sheet name="ATTEND" sheetId="9" r:id="rId2"/>
+    <sheet name="MISSION_DAILY" sheetId="2" r:id="rId3"/>
+    <sheet name="MISSION_PERIOD" sheetId="3" r:id="rId4"/>
+    <sheet name="ACHIEVE_ONCE" sheetId="4" r:id="rId5"/>
+    <sheet name="ACHIEVE_PASS" sheetId="5" r:id="rId6"/>
+    <sheet name="LEADERBOARD" sheetId="6" r:id="rId7"/>
+    <sheet name="LEADERBOARD_REWARD" sheetId="7" r:id="rId8"/>
+    <sheet name="ADVERTISE" sheetId="8" r:id="rId9"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="181">
   <si>
     <t>messageId</t>
   </si>
@@ -547,6 +548,36 @@
   </si>
   <si>
     <t>mission_period_02_005</t>
+  </si>
+  <si>
+    <t>day</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>attendId</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>attend_day_001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>attend_day_002</t>
+  </si>
+  <si>
+    <t>attend_day_003</t>
+  </si>
+  <si>
+    <t>attend_day_004</t>
+  </si>
+  <si>
+    <t>attend_day_005</t>
+  </si>
+  <si>
+    <t>attend_day_006</t>
+  </si>
+  <si>
+    <t>attend_day_007</t>
   </si>
 </sst>
 </file>
@@ -943,6 +974,7 @@
   <cols>
     <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1166,6 +1198,166 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F796D4AE-A38D-EF4C-BA92-C4794DD4EE94}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B10" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>180</v>
+      </c>
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -1382,7 +1574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
@@ -1706,7 +1898,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -2124,7 +2316,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -2487,7 +2679,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -2592,7 +2784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -2696,7 +2888,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>

</xml_diff>

<commit_message>
feature: ShopCatalogEvent 이벤트 상점 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/MetaTable.xlsx
+++ b/input/Domains/Game/MetaTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BDF27C-2DF1-534B-A6F6-BBE40A1B0502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9057882-F457-3742-9413-1039680E69C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ATTEND" sheetId="1" r:id="rId1"/>
@@ -1119,6 +1119,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="4" max="5" width="23" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
feature: PushManager 기능 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/MetaTable.xlsx
+++ b/input/Domains/Game/MetaTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F296F80-8C5C-544B-8D07-835ADD21AF50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5DCAD3-52CC-2C41-99EF-C0EB87613219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ADVERTISE" sheetId="8" r:id="rId1"/>
@@ -19,13 +19,27 @@
     <sheet name="LEADERBOARD_REWARD" sheetId="7" r:id="rId4"/>
     <sheet name="REWARD" sheetId="10" r:id="rId5"/>
     <sheet name="SEASON" sheetId="12" r:id="rId6"/>
+    <sheet name="PUSH" sheetId="13" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="120">
   <si>
     <t>attendId</t>
   </si>
@@ -359,6 +373,42 @@
   </si>
   <si>
     <t>reward_leaderboard_002</t>
+  </si>
+  <si>
+    <t>defaultMsg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>language</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>pushId</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Korean</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>English</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>group:true</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>string</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>event</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>topic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1519,4 +1569,78 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB9C5B22-DDA4-B440-BDB7-38839CB37699}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="2" width="12.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="str">
+        <f>LOWER(B5&amp;"_"&amp;C5)</f>
+        <v>event_korean</v>
+      </c>
+      <c r="B5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="str">
+        <f>LOWER(B6&amp;"_"&amp;C6)</f>
+        <v>event_english</v>
+      </c>
+      <c r="B6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feature: Operation에 push remote 전송 기능 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/MetaTable.xlsx
+++ b/input/Domains/Game/MetaTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5DCAD3-52CC-2C41-99EF-C0EB87613219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076E65AA-B1D5-774A-AE1A-924FF2EF1A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ADVERTISE" sheetId="8" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <sheet name="LEADERBOARD_REWARD" sheetId="7" r:id="rId4"/>
     <sheet name="REWARD" sheetId="10" r:id="rId5"/>
     <sheet name="SEASON" sheetId="12" r:id="rId6"/>
-    <sheet name="PUSH" sheetId="13" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="111">
   <si>
     <t>attendId</t>
   </si>
@@ -373,42 +372,6 @@
   </si>
   <si>
     <t>reward_leaderboard_002</t>
-  </si>
-  <si>
-    <t>defaultMsg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>language</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>pushId</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Korean</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>English</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>group:true</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>string</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>event</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>topic</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1569,78 +1532,4 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB9C5B22-DDA4-B440-BDB7-38839CB37699}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
-  <cols>
-    <col min="1" max="2" width="12.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="str">
-        <f>LOWER(B5&amp;"_"&amp;C5)</f>
-        <v>event_korean</v>
-      </c>
-      <c r="B5" t="s">
-        <v>118</v>
-      </c>
-      <c r="C5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="str">
-        <f>LOWER(B6&amp;"_"&amp;C6)</f>
-        <v>event_english</v>
-      </c>
-      <c r="B6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>